<commit_message>
feat: add premium images for all Refrigerados products and update excel database
</commit_message>
<xml_diff>
--- a/frontend/public/data/productos_inventario.xlsx
+++ b/frontend/public/data/productos_inventario.xlsx
@@ -2614,10 +2614,10 @@
       </c>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="n">
-        <v>18</v>
+        <v>88</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>388</v>
+        <v>268</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
@@ -2659,10 +2659,10 @@
       </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="n">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>163</v>
+        <v>300</v>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
@@ -2704,10 +2704,10 @@
       </c>
       <c r="I4" s="2" t="inlineStr"/>
       <c r="J4" s="2" t="n">
-        <v>14</v>
+        <v>93</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>315</v>
+        <v>332</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
@@ -2749,10 +2749,10 @@
       </c>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="n">
-        <v>73</v>
+        <v>51</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>477</v>
+        <v>147</v>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
@@ -2794,10 +2794,10 @@
       </c>
       <c r="I6" s="2" t="inlineStr"/>
       <c r="J6" s="2" t="n">
-        <v>44</v>
+        <v>18</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>427</v>
+        <v>94</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
@@ -2837,16 +2837,12 @@
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I7" s="2" t="inlineStr"/>
       <c r="J7" s="2" t="n">
-        <v>18</v>
+        <v>85</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>344</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
@@ -2888,10 +2884,10 @@
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="n">
-        <v>13</v>
+        <v>35</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>85</v>
+        <v>169</v>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
@@ -2931,12 +2927,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J9" s="2" t="n">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>321</v>
+        <v>330</v>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
@@ -2978,10 +2978,10 @@
       </c>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n">
-        <v>54</v>
+        <v>37</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>310</v>
+        <v>104</v>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
@@ -3023,10 +3023,10 @@
       </c>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>408</v>
+        <v>481</v>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
@@ -3066,12 +3066,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J12" s="2" t="n">
-        <v>43</v>
+        <v>80</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>199</v>
+        <v>224</v>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
@@ -3111,12 +3115,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J13" s="2" t="n">
-        <v>61</v>
+        <v>78</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>361</v>
+        <v>240</v>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
@@ -3158,10 +3166,10 @@
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="n">
-        <v>98</v>
+        <v>53</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>387</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
@@ -3203,10 +3211,10 @@
       </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="n">
-        <v>24</v>
+        <v>89</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>370</v>
+        <v>492</v>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
@@ -3246,16 +3254,12 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I16" s="2" t="inlineStr"/>
       <c r="J16" s="2" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>240</v>
+        <v>287</v>
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
@@ -3297,10 +3301,10 @@
       </c>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="n">
-        <v>67</v>
+        <v>93</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>256</v>
+        <v>399</v>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
@@ -3342,10 +3346,10 @@
       </c>
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="n">
-        <v>40</v>
+        <v>47</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>366</v>
+        <v>400</v>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
@@ -3387,10 +3391,10 @@
       </c>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="n">
-        <v>37</v>
+        <v>74</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>493</v>
+        <v>248</v>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
@@ -3430,16 +3434,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="n">
-        <v>91</v>
+        <v>52</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>74</v>
+        <v>403</v>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
@@ -3485,10 +3485,10 @@
         </is>
       </c>
       <c r="J21" s="2" t="n">
-        <v>48</v>
+        <v>97</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>274</v>
+        <v>338</v>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
@@ -3530,10 +3530,10 @@
       </c>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="n">
-        <v>50</v>
+        <v>100</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>292</v>
+        <v>97</v>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
@@ -3575,10 +3575,10 @@
       </c>
       <c r="I23" s="2" t="inlineStr"/>
       <c r="J23" s="2" t="n">
-        <v>95</v>
+        <v>25</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>102</v>
+        <v>163</v>
       </c>
     </row>
     <row r="24" ht="60" customHeight="1">
@@ -3620,10 +3620,10 @@
       </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="n">
-        <v>67</v>
+        <v>92</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>469</v>
+        <v>308</v>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
@@ -3665,10 +3665,10 @@
       </c>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="n">
-        <v>63</v>
+        <v>27</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>289</v>
+        <v>274</v>
       </c>
     </row>
     <row r="26" ht="60" customHeight="1">
@@ -3710,10 +3710,10 @@
       </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="n">
-        <v>67</v>
+        <v>87</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>499</v>
+        <v>396</v>
       </c>
     </row>
     <row r="27" ht="60" customHeight="1">
@@ -3755,10 +3755,10 @@
       </c>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="n">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>351</v>
+        <v>220</v>
       </c>
     </row>
     <row r="28" ht="60" customHeight="1">
@@ -3800,10 +3800,10 @@
       </c>
       <c r="I28" s="2" t="inlineStr"/>
       <c r="J28" s="2" t="n">
-        <v>20</v>
+        <v>98</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>253</v>
+        <v>112</v>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
@@ -3845,10 +3845,10 @@
       </c>
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="n">
-        <v>88</v>
+        <v>69</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>313</v>
+        <v>488</v>
       </c>
     </row>
     <row r="30" ht="60" customHeight="1">
@@ -3888,16 +3888,12 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="n">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>315</v>
+        <v>288</v>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
@@ -3937,16 +3933,12 @@
           <t>1 Paquete</t>
         </is>
       </c>
-      <c r="I31" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>161</v>
+        <v>367</v>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1">
@@ -3988,10 +3980,10 @@
       </c>
       <c r="I32" s="2" t="inlineStr"/>
       <c r="J32" s="2" t="n">
-        <v>71</v>
+        <v>93</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>60</v>
+        <v>331</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
@@ -4031,12 +4023,16 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J33" s="2" t="n">
-        <v>52</v>
+        <v>14</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>441</v>
+        <v>481</v>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1">
@@ -4076,16 +4072,12 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="n">
-        <v>77</v>
+        <v>14</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>208</v>
+        <v>356</v>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1">
@@ -4127,10 +4119,10 @@
       </c>
       <c r="I35" s="2" t="inlineStr"/>
       <c r="J35" s="2" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>487</v>
+        <v>442</v>
       </c>
     </row>
     <row r="36" ht="60" customHeight="1">
@@ -4172,10 +4164,10 @@
       </c>
       <c r="I36" s="2" t="inlineStr"/>
       <c r="J36" s="2" t="n">
-        <v>92</v>
+        <v>29</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>182</v>
+        <v>235</v>
       </c>
     </row>
     <row r="37" ht="60" customHeight="1">
@@ -4221,10 +4213,10 @@
         </is>
       </c>
       <c r="J37" s="2" t="n">
-        <v>57</v>
+        <v>16</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>354</v>
+        <v>52</v>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1">
@@ -4266,10 +4258,10 @@
       </c>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>203</v>
+        <v>433</v>
       </c>
     </row>
     <row r="39" ht="60" customHeight="1">
@@ -4309,12 +4301,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J39" s="2" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
       <c r="K39" s="2" t="n">
-        <v>52</v>
+        <v>143</v>
       </c>
     </row>
     <row r="40" ht="60" customHeight="1">
@@ -4354,16 +4350,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="n">
-        <v>23</v>
+        <v>79</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>338</v>
+        <v>66</v>
       </c>
     </row>
     <row r="41" ht="60" customHeight="1">
@@ -4403,12 +4395,16 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J41" s="2" t="n">
         <v>98</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>168</v>
+        <v>471</v>
       </c>
     </row>
     <row r="42" ht="60" customHeight="1">
@@ -4448,16 +4444,12 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="n">
-        <v>70</v>
+        <v>39</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>349</v>
+        <v>495</v>
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
@@ -4499,10 +4491,10 @@
       </c>
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="n">
-        <v>44</v>
+        <v>92</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>355</v>
+        <v>192</v>
       </c>
     </row>
     <row r="44" ht="60" customHeight="1">
@@ -4544,10 +4536,10 @@
       </c>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="n">
-        <v>77</v>
+        <v>29</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>294</v>
+        <v>139</v>
       </c>
     </row>
     <row r="45" ht="60" customHeight="1">
@@ -4587,16 +4579,12 @@
           <t>300g</t>
         </is>
       </c>
-      <c r="I45" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="2" t="n">
-        <v>96</v>
+        <v>62</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>82</v>
+        <v>148</v>
       </c>
     </row>
     <row r="46" ht="60" customHeight="1">
@@ -4638,10 +4626,10 @@
       </c>
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="n">
-        <v>98</v>
+        <v>19</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>252</v>
+        <v>341</v>
       </c>
     </row>
     <row r="47" ht="60" customHeight="1">
@@ -4683,10 +4671,10 @@
       </c>
       <c r="I47" s="2" t="inlineStr"/>
       <c r="J47" s="2" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>176</v>
+        <v>484</v>
       </c>
     </row>
     <row r="48" ht="60" customHeight="1">
@@ -4726,16 +4714,12 @@
           <t>50ml</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I48" s="2" t="inlineStr"/>
       <c r="J48" s="2" t="n">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>129</v>
+        <v>127</v>
       </c>
     </row>
     <row r="49" ht="60" customHeight="1">
@@ -4777,10 +4761,10 @@
       </c>
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="n">
-        <v>21</v>
+        <v>46</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>143</v>
+        <v>64</v>
       </c>
     </row>
     <row r="50" ht="60" customHeight="1">
@@ -4822,10 +4806,10 @@
       </c>
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="n">
-        <v>92</v>
+        <v>49</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>204</v>
+        <v>472</v>
       </c>
     </row>
     <row r="51" ht="60" customHeight="1">
@@ -4867,10 +4851,10 @@
       </c>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="n">
-        <v>51</v>
+        <v>87</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>138</v>
+        <v>180</v>
       </c>
     </row>
     <row r="52" ht="60" customHeight="1">
@@ -4912,10 +4896,10 @@
       </c>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="n">
-        <v>82</v>
+        <v>41</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>312</v>
+        <v>190</v>
       </c>
     </row>
     <row r="53" ht="60" customHeight="1">
@@ -4957,10 +4941,10 @@
       </c>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="n">
-        <v>70</v>
+        <v>20</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>380</v>
+        <v>229</v>
       </c>
     </row>
     <row r="54" ht="60" customHeight="1">
@@ -5002,10 +4986,10 @@
       </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="n">
-        <v>34</v>
+        <v>93</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>268</v>
+        <v>289</v>
       </c>
     </row>
     <row r="55" ht="60" customHeight="1">
@@ -5047,10 +5031,10 @@
       </c>
       <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="n">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>411</v>
+        <v>337</v>
       </c>
     </row>
     <row r="56" ht="60" customHeight="1">
@@ -5092,10 +5076,10 @@
       </c>
       <c r="I56" s="2" t="inlineStr"/>
       <c r="J56" s="2" t="n">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>374</v>
+        <v>280</v>
       </c>
     </row>
     <row r="57" ht="60" customHeight="1">
@@ -5135,16 +5119,12 @@
           <t>250ml</t>
         </is>
       </c>
-      <c r="I57" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="n">
-        <v>92</v>
+        <v>21</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>107</v>
+        <v>271</v>
       </c>
     </row>
     <row r="58" ht="60" customHeight="1">
@@ -5186,10 +5166,10 @@
       </c>
       <c r="I58" s="2" t="inlineStr"/>
       <c r="J58" s="2" t="n">
-        <v>94</v>
+        <v>69</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>422</v>
+        <v>157</v>
       </c>
     </row>
     <row r="59" ht="60" customHeight="1">
@@ -5231,10 +5211,10 @@
       </c>
       <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="2" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>102</v>
+        <v>74</v>
       </c>
     </row>
     <row r="60" ht="60" customHeight="1">
@@ -5274,16 +5254,12 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="I60" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="n">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>100</v>
+        <v>171</v>
       </c>
     </row>
     <row r="61" ht="60" customHeight="1">
@@ -5323,16 +5299,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I61" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I61" s="2" t="inlineStr"/>
       <c r="J61" s="2" t="n">
-        <v>75</v>
+        <v>44</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>459</v>
+        <v>173</v>
       </c>
     </row>
     <row r="62" ht="60" customHeight="1">
@@ -5374,10 +5346,10 @@
       </c>
       <c r="I62" s="2" t="inlineStr"/>
       <c r="J62" s="2" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>93</v>
+        <v>70</v>
       </c>
     </row>
     <row r="63" ht="60" customHeight="1">
@@ -5419,10 +5391,10 @@
       </c>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="n">
-        <v>96</v>
+        <v>43</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>369</v>
+        <v>475</v>
       </c>
     </row>
     <row r="64" ht="60" customHeight="1">
@@ -5464,10 +5436,10 @@
       </c>
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="n">
-        <v>98</v>
+        <v>13</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>364</v>
+        <v>252</v>
       </c>
     </row>
     <row r="65" ht="60" customHeight="1">
@@ -5509,10 +5481,10 @@
       </c>
       <c r="I65" s="2" t="inlineStr"/>
       <c r="J65" s="2" t="n">
-        <v>55</v>
+        <v>99</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>206</v>
+        <v>136</v>
       </c>
     </row>
     <row r="66" ht="60" customHeight="1">
@@ -5554,10 +5526,10 @@
       </c>
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="n">
-        <v>24</v>
+        <v>50</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>321</v>
+        <v>487</v>
       </c>
     </row>
     <row r="67" ht="60" customHeight="1">
@@ -5599,10 +5571,10 @@
       </c>
       <c r="I67" s="2" t="inlineStr"/>
       <c r="J67" s="2" t="n">
-        <v>21</v>
+        <v>36</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>65</v>
+        <v>161</v>
       </c>
     </row>
     <row r="68" ht="60" customHeight="1">
@@ -5644,10 +5616,10 @@
       </c>
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="n">
-        <v>78</v>
+        <v>44</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>276</v>
+        <v>253</v>
       </c>
     </row>
     <row r="69" ht="60" customHeight="1">
@@ -5687,12 +5659,16 @@
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J69" s="2" t="n">
-        <v>47</v>
+        <v>87</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>323</v>
+        <v>113</v>
       </c>
     </row>
     <row r="70" ht="60" customHeight="1">
@@ -5734,10 +5710,10 @@
       </c>
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="n">
-        <v>92</v>
+        <v>48</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>161</v>
+        <v>175</v>
       </c>
     </row>
     <row r="71" ht="60" customHeight="1">
@@ -5777,16 +5753,12 @@
           <t>10 Unidades</t>
         </is>
       </c>
-      <c r="I71" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="n">
-        <v>100</v>
+        <v>92</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>421</v>
+        <v>387</v>
       </c>
     </row>
     <row r="72" ht="60" customHeight="1">
@@ -5826,16 +5798,12 @@
           <t>Caja 36</t>
         </is>
       </c>
-      <c r="I72" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="n">
-        <v>96</v>
+        <v>14</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>235</v>
+        <v>224</v>
       </c>
     </row>
     <row r="73" ht="60" customHeight="1">
@@ -5877,10 +5845,10 @@
       </c>
       <c r="I73" s="2" t="inlineStr"/>
       <c r="J73" s="2" t="n">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>144</v>
+        <v>497</v>
       </c>
     </row>
     <row r="74" ht="60" customHeight="1">
@@ -5922,10 +5890,10 @@
       </c>
       <c r="I74" s="2" t="inlineStr"/>
       <c r="J74" s="2" t="n">
-        <v>15</v>
+        <v>84</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>238</v>
+        <v>205</v>
       </c>
     </row>
     <row r="75" ht="60" customHeight="1">
@@ -5967,10 +5935,10 @@
       </c>
       <c r="I75" s="2" t="inlineStr"/>
       <c r="J75" s="2" t="n">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>314</v>
+        <v>325</v>
       </c>
     </row>
     <row r="76" ht="60" customHeight="1">
@@ -6012,10 +5980,10 @@
       </c>
       <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="n">
-        <v>14</v>
+        <v>93</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>241</v>
+        <v>56</v>
       </c>
     </row>
     <row r="77" ht="60" customHeight="1">
@@ -6055,16 +6023,12 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I77" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I77" s="2" t="inlineStr"/>
       <c r="J77" s="2" t="n">
-        <v>24</v>
+        <v>58</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>415</v>
+        <v>261</v>
       </c>
     </row>
     <row r="78" ht="60" customHeight="1">
@@ -6106,10 +6070,10 @@
       </c>
       <c r="I78" s="2" t="inlineStr"/>
       <c r="J78" s="2" t="n">
-        <v>29</v>
+        <v>61</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>160</v>
+        <v>281</v>
       </c>
     </row>
     <row r="79" ht="60" customHeight="1">
@@ -6151,10 +6115,10 @@
       </c>
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="n">
-        <v>34</v>
+        <v>15</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>338</v>
+        <v>226</v>
       </c>
     </row>
     <row r="80" ht="60" customHeight="1">
@@ -6196,10 +6160,10 @@
       </c>
       <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="n">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>54</v>
+        <v>476</v>
       </c>
     </row>
     <row r="81" ht="60" customHeight="1">
@@ -6239,16 +6203,12 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I81" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I81" s="2" t="inlineStr"/>
       <c r="J81" s="2" t="n">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>313</v>
+        <v>132</v>
       </c>
     </row>
     <row r="82" ht="60" customHeight="1">
@@ -6288,16 +6248,12 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I82" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="n">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="K82" s="2" t="n">
-        <v>260</v>
+        <v>470</v>
       </c>
     </row>
     <row r="83" ht="60" customHeight="1">
@@ -6339,14 +6295,14 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>Oferta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="J83" s="2" t="n">
-        <v>36</v>
+        <v>58</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>81</v>
+        <v>479</v>
       </c>
     </row>
     <row r="84" ht="60" customHeight="1">
@@ -6388,10 +6344,10 @@
       </c>
       <c r="I84" s="2" t="inlineStr"/>
       <c r="J84" s="2" t="n">
-        <v>82</v>
+        <v>23</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>108</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: batch remove background and apply pure white background for all 83 products
</commit_message>
<xml_diff>
--- a/frontend/public/data/productos_inventario.xlsx
+++ b/frontend/public/data/productos_inventario.xlsx
@@ -2614,10 +2614,10 @@
       </c>
       <c r="I2" s="2" t="inlineStr"/>
       <c r="J2" s="2" t="n">
-        <v>88</v>
+        <v>60</v>
       </c>
       <c r="K2" s="2" t="n">
-        <v>268</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" ht="60" customHeight="1">
@@ -2659,10 +2659,10 @@
       </c>
       <c r="I3" s="2" t="inlineStr"/>
       <c r="J3" s="2" t="n">
-        <v>56</v>
+        <v>75</v>
       </c>
       <c r="K3" s="2" t="n">
-        <v>300</v>
+        <v>497</v>
       </c>
     </row>
     <row r="4" ht="60" customHeight="1">
@@ -2702,12 +2702,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J4" s="2" t="n">
-        <v>93</v>
+        <v>13</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>332</v>
+        <v>276</v>
       </c>
     </row>
     <row r="5" ht="60" customHeight="1">
@@ -2749,10 +2753,10 @@
       </c>
       <c r="I5" s="2" t="inlineStr"/>
       <c r="J5" s="2" t="n">
-        <v>51</v>
+        <v>16</v>
       </c>
       <c r="K5" s="2" t="n">
-        <v>147</v>
+        <v>276</v>
       </c>
     </row>
     <row r="6" ht="60" customHeight="1">
@@ -2792,12 +2796,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J6" s="2" t="n">
-        <v>18</v>
+        <v>51</v>
       </c>
       <c r="K6" s="2" t="n">
-        <v>94</v>
+        <v>477</v>
       </c>
     </row>
     <row r="7" ht="60" customHeight="1">
@@ -2837,12 +2845,16 @@
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="I7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J7" s="2" t="n">
         <v>85</v>
       </c>
       <c r="K7" s="2" t="n">
-        <v>67</v>
+        <v>458</v>
       </c>
     </row>
     <row r="8" ht="60" customHeight="1">
@@ -2884,10 +2896,10 @@
       </c>
       <c r="I8" s="2" t="inlineStr"/>
       <c r="J8" s="2" t="n">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="K8" s="2" t="n">
-        <v>169</v>
+        <v>313</v>
       </c>
     </row>
     <row r="9" ht="60" customHeight="1">
@@ -2927,16 +2939,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I9" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I9" s="2" t="inlineStr"/>
       <c r="J9" s="2" t="n">
-        <v>25</v>
+        <v>68</v>
       </c>
       <c r="K9" s="2" t="n">
-        <v>330</v>
+        <v>128</v>
       </c>
     </row>
     <row r="10" ht="60" customHeight="1">
@@ -2978,10 +2986,10 @@
       </c>
       <c r="I10" s="2" t="inlineStr"/>
       <c r="J10" s="2" t="n">
-        <v>37</v>
+        <v>60</v>
       </c>
       <c r="K10" s="2" t="n">
-        <v>104</v>
+        <v>336</v>
       </c>
     </row>
     <row r="11" ht="60" customHeight="1">
@@ -3023,10 +3031,10 @@
       </c>
       <c r="I11" s="2" t="inlineStr"/>
       <c r="J11" s="2" t="n">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="K11" s="2" t="n">
-        <v>481</v>
+        <v>417</v>
       </c>
     </row>
     <row r="12" ht="60" customHeight="1">
@@ -3066,16 +3074,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I12" s="2" t="inlineStr"/>
       <c r="J12" s="2" t="n">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="K12" s="2" t="n">
-        <v>224</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" ht="60" customHeight="1">
@@ -3115,16 +3119,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I13" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I13" s="2" t="inlineStr"/>
       <c r="J13" s="2" t="n">
-        <v>78</v>
+        <v>29</v>
       </c>
       <c r="K13" s="2" t="n">
-        <v>240</v>
+        <v>109</v>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
@@ -3166,10 +3166,10 @@
       </c>
       <c r="I14" s="2" t="inlineStr"/>
       <c r="J14" s="2" t="n">
-        <v>53</v>
+        <v>38</v>
       </c>
       <c r="K14" s="2" t="n">
-        <v>262</v>
+        <v>340</v>
       </c>
     </row>
     <row r="15" ht="60" customHeight="1">
@@ -3211,10 +3211,10 @@
       </c>
       <c r="I15" s="2" t="inlineStr"/>
       <c r="J15" s="2" t="n">
-        <v>89</v>
+        <v>53</v>
       </c>
       <c r="K15" s="2" t="n">
-        <v>492</v>
+        <v>486</v>
       </c>
     </row>
     <row r="16" ht="60" customHeight="1">
@@ -3254,12 +3254,16 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J16" s="2" t="n">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="K16" s="2" t="n">
-        <v>287</v>
+        <v>384</v>
       </c>
     </row>
     <row r="17" ht="60" customHeight="1">
@@ -3301,10 +3305,10 @@
       </c>
       <c r="I17" s="2" t="inlineStr"/>
       <c r="J17" s="2" t="n">
-        <v>93</v>
+        <v>78</v>
       </c>
       <c r="K17" s="2" t="n">
-        <v>399</v>
+        <v>271</v>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
@@ -3346,10 +3350,10 @@
       </c>
       <c r="I18" s="2" t="inlineStr"/>
       <c r="J18" s="2" t="n">
-        <v>47</v>
+        <v>62</v>
       </c>
       <c r="K18" s="2" t="n">
-        <v>400</v>
+        <v>399</v>
       </c>
     </row>
     <row r="19" ht="60" customHeight="1">
@@ -3391,10 +3395,10 @@
       </c>
       <c r="I19" s="2" t="inlineStr"/>
       <c r="J19" s="2" t="n">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="K19" s="2" t="n">
-        <v>248</v>
+        <v>253</v>
       </c>
     </row>
     <row r="20" ht="60" customHeight="1">
@@ -3436,10 +3440,10 @@
       </c>
       <c r="I20" s="2" t="inlineStr"/>
       <c r="J20" s="2" t="n">
-        <v>52</v>
+        <v>38</v>
       </c>
       <c r="K20" s="2" t="n">
-        <v>403</v>
+        <v>158</v>
       </c>
     </row>
     <row r="21" ht="60" customHeight="1">
@@ -3479,16 +3483,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I21" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I21" s="2" t="inlineStr"/>
       <c r="J21" s="2" t="n">
-        <v>97</v>
+        <v>90</v>
       </c>
       <c r="K21" s="2" t="n">
-        <v>338</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22" ht="60" customHeight="1">
@@ -3530,10 +3530,10 @@
       </c>
       <c r="I22" s="2" t="inlineStr"/>
       <c r="J22" s="2" t="n">
-        <v>100</v>
+        <v>90</v>
       </c>
       <c r="K22" s="2" t="n">
-        <v>97</v>
+        <v>472</v>
       </c>
     </row>
     <row r="23" ht="60" customHeight="1">
@@ -3573,12 +3573,16 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J23" s="2" t="n">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="K23" s="2" t="n">
-        <v>163</v>
+        <v>287</v>
       </c>
     </row>
     <row r="24" ht="60" customHeight="1">
@@ -3620,10 +3624,10 @@
       </c>
       <c r="I24" s="2" t="inlineStr"/>
       <c r="J24" s="2" t="n">
-        <v>92</v>
+        <v>56</v>
       </c>
       <c r="K24" s="2" t="n">
-        <v>308</v>
+        <v>454</v>
       </c>
     </row>
     <row r="25" ht="60" customHeight="1">
@@ -3665,10 +3669,10 @@
       </c>
       <c r="I25" s="2" t="inlineStr"/>
       <c r="J25" s="2" t="n">
-        <v>27</v>
+        <v>73</v>
       </c>
       <c r="K25" s="2" t="n">
-        <v>274</v>
+        <v>419</v>
       </c>
     </row>
     <row r="26" ht="60" customHeight="1">
@@ -3710,10 +3714,10 @@
       </c>
       <c r="I26" s="2" t="inlineStr"/>
       <c r="J26" s="2" t="n">
-        <v>87</v>
+        <v>45</v>
       </c>
       <c r="K26" s="2" t="n">
-        <v>396</v>
+        <v>457</v>
       </c>
     </row>
     <row r="27" ht="60" customHeight="1">
@@ -3755,10 +3759,10 @@
       </c>
       <c r="I27" s="2" t="inlineStr"/>
       <c r="J27" s="2" t="n">
-        <v>96</v>
+        <v>84</v>
       </c>
       <c r="K27" s="2" t="n">
-        <v>220</v>
+        <v>296</v>
       </c>
     </row>
     <row r="28" ht="60" customHeight="1">
@@ -3798,12 +3802,16 @@
           <t>250g</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J28" s="2" t="n">
-        <v>98</v>
+        <v>55</v>
       </c>
       <c r="K28" s="2" t="n">
-        <v>112</v>
+        <v>162</v>
       </c>
     </row>
     <row r="29" ht="60" customHeight="1">
@@ -3845,10 +3853,10 @@
       </c>
       <c r="I29" s="2" t="inlineStr"/>
       <c r="J29" s="2" t="n">
-        <v>69</v>
+        <v>28</v>
       </c>
       <c r="K29" s="2" t="n">
-        <v>488</v>
+        <v>157</v>
       </c>
     </row>
     <row r="30" ht="60" customHeight="1">
@@ -3890,10 +3898,10 @@
       </c>
       <c r="I30" s="2" t="inlineStr"/>
       <c r="J30" s="2" t="n">
-        <v>83</v>
+        <v>47</v>
       </c>
       <c r="K30" s="2" t="n">
-        <v>288</v>
+        <v>220</v>
       </c>
     </row>
     <row r="31" ht="60" customHeight="1">
@@ -3935,10 +3943,10 @@
       </c>
       <c r="I31" s="2" t="inlineStr"/>
       <c r="J31" s="2" t="n">
-        <v>78</v>
+        <v>98</v>
       </c>
       <c r="K31" s="2" t="n">
-        <v>367</v>
+        <v>95</v>
       </c>
     </row>
     <row r="32" ht="60" customHeight="1">
@@ -3978,12 +3986,16 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J32" s="2" t="n">
-        <v>93</v>
+        <v>61</v>
       </c>
       <c r="K32" s="2" t="n">
-        <v>331</v>
+        <v>309</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
@@ -4023,16 +4035,12 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="I33" s="2" t="inlineStr">
-        <is>
-          <t>Oferta</t>
-        </is>
-      </c>
+      <c r="I33" s="2" t="inlineStr"/>
       <c r="J33" s="2" t="n">
-        <v>14</v>
+        <v>32</v>
       </c>
       <c r="K33" s="2" t="n">
-        <v>481</v>
+        <v>427</v>
       </c>
     </row>
     <row r="34" ht="60" customHeight="1">
@@ -4074,10 +4082,10 @@
       </c>
       <c r="I34" s="2" t="inlineStr"/>
       <c r="J34" s="2" t="n">
-        <v>14</v>
+        <v>85</v>
       </c>
       <c r="K34" s="2" t="n">
-        <v>356</v>
+        <v>193</v>
       </c>
     </row>
     <row r="35" ht="60" customHeight="1">
@@ -4117,12 +4125,16 @@
           <t>2 L</t>
         </is>
       </c>
-      <c r="I35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J35" s="2" t="n">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="K35" s="2" t="n">
-        <v>442</v>
+        <v>446</v>
       </c>
     </row>
     <row r="36" ht="60" customHeight="1">
@@ -4162,12 +4174,16 @@
           <t>1.5 L</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J36" s="2" t="n">
-        <v>29</v>
+        <v>19</v>
       </c>
       <c r="K36" s="2" t="n">
-        <v>235</v>
+        <v>257</v>
       </c>
     </row>
     <row r="37" ht="60" customHeight="1">
@@ -4207,16 +4223,12 @@
           <t>1 Kg</t>
         </is>
       </c>
-      <c r="I37" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I37" s="2" t="inlineStr"/>
       <c r="J37" s="2" t="n">
-        <v>16</v>
+        <v>86</v>
       </c>
       <c r="K37" s="2" t="n">
-        <v>52</v>
+        <v>294</v>
       </c>
     </row>
     <row r="38" ht="60" customHeight="1">
@@ -4258,10 +4270,10 @@
       </c>
       <c r="I38" s="2" t="inlineStr"/>
       <c r="J38" s="2" t="n">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="K38" s="2" t="n">
-        <v>433</v>
+        <v>443</v>
       </c>
     </row>
     <row r="39" ht="60" customHeight="1">
@@ -4303,14 +4315,14 @@
       </c>
       <c r="I39" s="2" t="inlineStr">
         <is>
-          <t>Oferta</t>
+          <t>Nuevo</t>
         </is>
       </c>
       <c r="J39" s="2" t="n">
+        <v>63</v>
+      </c>
+      <c r="K39" s="2" t="n">
         <v>72</v>
-      </c>
-      <c r="K39" s="2" t="n">
-        <v>143</v>
       </c>
     </row>
     <row r="40" ht="60" customHeight="1">
@@ -4352,10 +4364,10 @@
       </c>
       <c r="I40" s="2" t="inlineStr"/>
       <c r="J40" s="2" t="n">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="K40" s="2" t="n">
-        <v>66</v>
+        <v>96</v>
       </c>
     </row>
     <row r="41" ht="60" customHeight="1">
@@ -4395,16 +4407,12 @@
           <t>500g</t>
         </is>
       </c>
-      <c r="I41" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I41" s="2" t="inlineStr"/>
       <c r="J41" s="2" t="n">
-        <v>98</v>
+        <v>37</v>
       </c>
       <c r="K41" s="2" t="n">
-        <v>471</v>
+        <v>149</v>
       </c>
     </row>
     <row r="42" ht="60" customHeight="1">
@@ -4446,10 +4454,10 @@
       </c>
       <c r="I42" s="2" t="inlineStr"/>
       <c r="J42" s="2" t="n">
-        <v>39</v>
+        <v>74</v>
       </c>
       <c r="K42" s="2" t="n">
-        <v>495</v>
+        <v>197</v>
       </c>
     </row>
     <row r="43" ht="60" customHeight="1">
@@ -4491,10 +4499,10 @@
       </c>
       <c r="I43" s="2" t="inlineStr"/>
       <c r="J43" s="2" t="n">
-        <v>92</v>
+        <v>73</v>
       </c>
       <c r="K43" s="2" t="n">
-        <v>192</v>
+        <v>162</v>
       </c>
     </row>
     <row r="44" ht="60" customHeight="1">
@@ -4536,10 +4544,10 @@
       </c>
       <c r="I44" s="2" t="inlineStr"/>
       <c r="J44" s="2" t="n">
-        <v>29</v>
+        <v>68</v>
       </c>
       <c r="K44" s="2" t="n">
-        <v>139</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" ht="60" customHeight="1">
@@ -4581,10 +4589,10 @@
       </c>
       <c r="I45" s="2" t="inlineStr"/>
       <c r="J45" s="2" t="n">
-        <v>62</v>
+        <v>100</v>
       </c>
       <c r="K45" s="2" t="n">
-        <v>148</v>
+        <v>193</v>
       </c>
     </row>
     <row r="46" ht="60" customHeight="1">
@@ -4626,10 +4634,10 @@
       </c>
       <c r="I46" s="2" t="inlineStr"/>
       <c r="J46" s="2" t="n">
-        <v>19</v>
+        <v>95</v>
       </c>
       <c r="K46" s="2" t="n">
-        <v>341</v>
+        <v>237</v>
       </c>
     </row>
     <row r="47" ht="60" customHeight="1">
@@ -4669,12 +4677,16 @@
           <t>3 Unidades</t>
         </is>
       </c>
-      <c r="I47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J47" s="2" t="n">
-        <v>60</v>
+        <v>94</v>
       </c>
       <c r="K47" s="2" t="n">
-        <v>484</v>
+        <v>302</v>
       </c>
     </row>
     <row r="48" ht="60" customHeight="1">
@@ -4714,12 +4726,16 @@
           <t>50ml</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J48" s="2" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="K48" s="2" t="n">
-        <v>127</v>
+        <v>363</v>
       </c>
     </row>
     <row r="49" ht="60" customHeight="1">
@@ -4761,10 +4777,10 @@
       </c>
       <c r="I49" s="2" t="inlineStr"/>
       <c r="J49" s="2" t="n">
-        <v>46</v>
+        <v>58</v>
       </c>
       <c r="K49" s="2" t="n">
-        <v>64</v>
+        <v>108</v>
       </c>
     </row>
     <row r="50" ht="60" customHeight="1">
@@ -4806,10 +4822,10 @@
       </c>
       <c r="I50" s="2" t="inlineStr"/>
       <c r="J50" s="2" t="n">
-        <v>49</v>
+        <v>58</v>
       </c>
       <c r="K50" s="2" t="n">
-        <v>472</v>
+        <v>55</v>
       </c>
     </row>
     <row r="51" ht="60" customHeight="1">
@@ -4851,10 +4867,10 @@
       </c>
       <c r="I51" s="2" t="inlineStr"/>
       <c r="J51" s="2" t="n">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="K51" s="2" t="n">
-        <v>180</v>
+        <v>372</v>
       </c>
     </row>
     <row r="52" ht="60" customHeight="1">
@@ -4896,10 +4912,10 @@
       </c>
       <c r="I52" s="2" t="inlineStr"/>
       <c r="J52" s="2" t="n">
-        <v>41</v>
+        <v>92</v>
       </c>
       <c r="K52" s="2" t="n">
-        <v>190</v>
+        <v>113</v>
       </c>
     </row>
     <row r="53" ht="60" customHeight="1">
@@ -4941,10 +4957,10 @@
       </c>
       <c r="I53" s="2" t="inlineStr"/>
       <c r="J53" s="2" t="n">
-        <v>20</v>
+        <v>90</v>
       </c>
       <c r="K53" s="2" t="n">
-        <v>229</v>
+        <v>312</v>
       </c>
     </row>
     <row r="54" ht="60" customHeight="1">
@@ -4986,10 +5002,10 @@
       </c>
       <c r="I54" s="2" t="inlineStr"/>
       <c r="J54" s="2" t="n">
-        <v>93</v>
+        <v>40</v>
       </c>
       <c r="K54" s="2" t="n">
-        <v>289</v>
+        <v>189</v>
       </c>
     </row>
     <row r="55" ht="60" customHeight="1">
@@ -5031,10 +5047,10 @@
       </c>
       <c r="I55" s="2" t="inlineStr"/>
       <c r="J55" s="2" t="n">
-        <v>94</v>
+        <v>35</v>
       </c>
       <c r="K55" s="2" t="n">
-        <v>337</v>
+        <v>192</v>
       </c>
     </row>
     <row r="56" ht="60" customHeight="1">
@@ -5074,12 +5090,16 @@
           <t>100 Unidades</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J56" s="2" t="n">
-        <v>29</v>
+        <v>90</v>
       </c>
       <c r="K56" s="2" t="n">
-        <v>280</v>
+        <v>55</v>
       </c>
     </row>
     <row r="57" ht="60" customHeight="1">
@@ -5121,10 +5141,10 @@
       </c>
       <c r="I57" s="2" t="inlineStr"/>
       <c r="J57" s="2" t="n">
-        <v>21</v>
+        <v>45</v>
       </c>
       <c r="K57" s="2" t="n">
-        <v>271</v>
+        <v>372</v>
       </c>
     </row>
     <row r="58" ht="60" customHeight="1">
@@ -5164,12 +5184,16 @@
           <t>100ml</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J58" s="2" t="n">
-        <v>69</v>
+        <v>14</v>
       </c>
       <c r="K58" s="2" t="n">
-        <v>157</v>
+        <v>284</v>
       </c>
     </row>
     <row r="59" ht="60" customHeight="1">
@@ -5211,10 +5235,10 @@
       </c>
       <c r="I59" s="2" t="inlineStr"/>
       <c r="J59" s="2" t="n">
-        <v>73</v>
+        <v>89</v>
       </c>
       <c r="K59" s="2" t="n">
-        <v>74</v>
+        <v>341</v>
       </c>
     </row>
     <row r="60" ht="60" customHeight="1">
@@ -5256,10 +5280,10 @@
       </c>
       <c r="I60" s="2" t="inlineStr"/>
       <c r="J60" s="2" t="n">
-        <v>40</v>
+        <v>50</v>
       </c>
       <c r="K60" s="2" t="n">
-        <v>171</v>
+        <v>131</v>
       </c>
     </row>
     <row r="61" ht="60" customHeight="1">
@@ -5301,10 +5325,10 @@
       </c>
       <c r="I61" s="2" t="inlineStr"/>
       <c r="J61" s="2" t="n">
-        <v>44</v>
+        <v>90</v>
       </c>
       <c r="K61" s="2" t="n">
-        <v>173</v>
+        <v>313</v>
       </c>
     </row>
     <row r="62" ht="60" customHeight="1">
@@ -5344,12 +5368,16 @@
           <t>1 L</t>
         </is>
       </c>
-      <c r="I62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J62" s="2" t="n">
-        <v>50</v>
+        <v>72</v>
       </c>
       <c r="K62" s="2" t="n">
-        <v>70</v>
+        <v>446</v>
       </c>
     </row>
     <row r="63" ht="60" customHeight="1">
@@ -5391,10 +5419,10 @@
       </c>
       <c r="I63" s="2" t="inlineStr"/>
       <c r="J63" s="2" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="K63" s="2" t="n">
-        <v>475</v>
+        <v>363</v>
       </c>
     </row>
     <row r="64" ht="60" customHeight="1">
@@ -5436,10 +5464,10 @@
       </c>
       <c r="I64" s="2" t="inlineStr"/>
       <c r="J64" s="2" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="K64" s="2" t="n">
-        <v>252</v>
+        <v>427</v>
       </c>
     </row>
     <row r="65" ht="60" customHeight="1">
@@ -5481,10 +5509,10 @@
       </c>
       <c r="I65" s="2" t="inlineStr"/>
       <c r="J65" s="2" t="n">
-        <v>99</v>
+        <v>83</v>
       </c>
       <c r="K65" s="2" t="n">
-        <v>136</v>
+        <v>272</v>
       </c>
     </row>
     <row r="66" ht="60" customHeight="1">
@@ -5526,10 +5554,10 @@
       </c>
       <c r="I66" s="2" t="inlineStr"/>
       <c r="J66" s="2" t="n">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="K66" s="2" t="n">
-        <v>487</v>
+        <v>435</v>
       </c>
     </row>
     <row r="67" ht="60" customHeight="1">
@@ -5569,12 +5597,16 @@
           <t>3 Unidades</t>
         </is>
       </c>
-      <c r="I67" s="2" t="inlineStr"/>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J67" s="2" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="K67" s="2" t="n">
-        <v>161</v>
+        <v>456</v>
       </c>
     </row>
     <row r="68" ht="60" customHeight="1">
@@ -5616,10 +5648,10 @@
       </c>
       <c r="I68" s="2" t="inlineStr"/>
       <c r="J68" s="2" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="K68" s="2" t="n">
-        <v>253</v>
+        <v>137</v>
       </c>
     </row>
     <row r="69" ht="60" customHeight="1">
@@ -5659,16 +5691,12 @@
           <t>1 Unidad</t>
         </is>
       </c>
-      <c r="I69" s="2" t="inlineStr">
-        <is>
-          <t>Nuevo</t>
-        </is>
-      </c>
+      <c r="I69" s="2" t="inlineStr"/>
       <c r="J69" s="2" t="n">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="K69" s="2" t="n">
-        <v>113</v>
+        <v>328</v>
       </c>
     </row>
     <row r="70" ht="60" customHeight="1">
@@ -5710,10 +5738,10 @@
       </c>
       <c r="I70" s="2" t="inlineStr"/>
       <c r="J70" s="2" t="n">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="K70" s="2" t="n">
-        <v>175</v>
+        <v>288</v>
       </c>
     </row>
     <row r="71" ht="60" customHeight="1">
@@ -5755,10 +5783,10 @@
       </c>
       <c r="I71" s="2" t="inlineStr"/>
       <c r="J71" s="2" t="n">
-        <v>92</v>
+        <v>81</v>
       </c>
       <c r="K71" s="2" t="n">
-        <v>387</v>
+        <v>208</v>
       </c>
     </row>
     <row r="72" ht="60" customHeight="1">
@@ -5800,10 +5828,10 @@
       </c>
       <c r="I72" s="2" t="inlineStr"/>
       <c r="J72" s="2" t="n">
-        <v>14</v>
+        <v>41</v>
       </c>
       <c r="K72" s="2" t="n">
-        <v>224</v>
+        <v>102</v>
       </c>
     </row>
     <row r="73" ht="60" customHeight="1">
@@ -5845,10 +5873,10 @@
       </c>
       <c r="I73" s="2" t="inlineStr"/>
       <c r="J73" s="2" t="n">
-        <v>65</v>
+        <v>21</v>
       </c>
       <c r="K73" s="2" t="n">
-        <v>497</v>
+        <v>492</v>
       </c>
     </row>
     <row r="74" ht="60" customHeight="1">
@@ -5888,12 +5916,16 @@
           <t>6 Pack</t>
         </is>
       </c>
-      <c r="I74" s="2" t="inlineStr"/>
+      <c r="I74" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J74" s="2" t="n">
-        <v>84</v>
+        <v>28</v>
       </c>
       <c r="K74" s="2" t="n">
-        <v>205</v>
+        <v>50</v>
       </c>
     </row>
     <row r="75" ht="60" customHeight="1">
@@ -5935,10 +5967,10 @@
       </c>
       <c r="I75" s="2" t="inlineStr"/>
       <c r="J75" s="2" t="n">
-        <v>41</v>
+        <v>86</v>
       </c>
       <c r="K75" s="2" t="n">
-        <v>325</v>
+        <v>73</v>
       </c>
     </row>
     <row r="76" ht="60" customHeight="1">
@@ -5980,10 +6012,10 @@
       </c>
       <c r="I76" s="2" t="inlineStr"/>
       <c r="J76" s="2" t="n">
-        <v>93</v>
+        <v>81</v>
       </c>
       <c r="K76" s="2" t="n">
-        <v>56</v>
+        <v>392</v>
       </c>
     </row>
     <row r="77" ht="60" customHeight="1">
@@ -6025,10 +6057,10 @@
       </c>
       <c r="I77" s="2" t="inlineStr"/>
       <c r="J77" s="2" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="K77" s="2" t="n">
-        <v>261</v>
+        <v>366</v>
       </c>
     </row>
     <row r="78" ht="60" customHeight="1">
@@ -6070,10 +6102,10 @@
       </c>
       <c r="I78" s="2" t="inlineStr"/>
       <c r="J78" s="2" t="n">
-        <v>61</v>
+        <v>74</v>
       </c>
       <c r="K78" s="2" t="n">
-        <v>281</v>
+        <v>334</v>
       </c>
     </row>
     <row r="79" ht="60" customHeight="1">
@@ -6115,10 +6147,10 @@
       </c>
       <c r="I79" s="2" t="inlineStr"/>
       <c r="J79" s="2" t="n">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="K79" s="2" t="n">
-        <v>226</v>
+        <v>50</v>
       </c>
     </row>
     <row r="80" ht="60" customHeight="1">
@@ -6160,10 +6192,10 @@
       </c>
       <c r="I80" s="2" t="inlineStr"/>
       <c r="J80" s="2" t="n">
-        <v>80</v>
+        <v>28</v>
       </c>
       <c r="K80" s="2" t="n">
-        <v>476</v>
+        <v>170</v>
       </c>
     </row>
     <row r="81" ht="60" customHeight="1">
@@ -6203,12 +6235,16 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I81" s="2" t="inlineStr"/>
+      <c r="I81" s="2" t="inlineStr">
+        <is>
+          <t>Nuevo</t>
+        </is>
+      </c>
       <c r="J81" s="2" t="n">
-        <v>84</v>
+        <v>77</v>
       </c>
       <c r="K81" s="2" t="n">
-        <v>132</v>
+        <v>274</v>
       </c>
     </row>
     <row r="82" ht="60" customHeight="1">
@@ -6250,10 +6286,10 @@
       </c>
       <c r="I82" s="2" t="inlineStr"/>
       <c r="J82" s="2" t="n">
+        <v>82</v>
+      </c>
+      <c r="K82" s="2" t="n">
         <v>52</v>
-      </c>
-      <c r="K82" s="2" t="n">
-        <v>470</v>
       </c>
     </row>
     <row r="83" ht="60" customHeight="1">
@@ -6295,14 +6331,14 @@
       </c>
       <c r="I83" s="2" t="inlineStr">
         <is>
-          <t>Nuevo</t>
+          <t>Oferta</t>
         </is>
       </c>
       <c r="J83" s="2" t="n">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="K83" s="2" t="n">
-        <v>479</v>
+        <v>498</v>
       </c>
     </row>
     <row r="84" ht="60" customHeight="1">
@@ -6342,12 +6378,16 @@
           <t>750ml</t>
         </is>
       </c>
-      <c r="I84" s="2" t="inlineStr"/>
+      <c r="I84" s="2" t="inlineStr">
+        <is>
+          <t>Oferta</t>
+        </is>
+      </c>
       <c r="J84" s="2" t="n">
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="K84" s="2" t="n">
-        <v>73</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Manually override subcategories for Harina, Aceites, and Granos, and restore names/prices for incorrect El Plazas search matches
</commit_message>
<xml_diff>
--- a/frontend/public/data/productos_inventario.xlsx
+++ b/frontend/public/data/productos_inventario.xlsx
@@ -2879,11 +2879,11 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>CEBOLLA INDIAN MOLIDA 55G</t>
+          <t>Cebolla Blanca X KG</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
-        <v>3.29</v>
+        <v>2.1</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -3055,11 +3055,11 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>LECHUGA ROMANA CULPROFRES 450G</t>
+          <t>Lechuga Romana</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
-        <v>2.95</v>
+        <v>1.2</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -3677,11 +3677,11 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>POLLO ENTERO UN POLLO PREMIUM X KG</t>
+          <t>Pollo Entero X KG</t>
         </is>
       </c>
       <c r="C21" s="2" t="n">
-        <v>4.45</v>
+        <v>4.5</v>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
@@ -3767,11 +3767,11 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>DIADEX CREMA ANTIPAÑALITIS ALOE TUBO 50G</t>
+          <t>Alitas de Pollo X KG</t>
         </is>
       </c>
       <c r="C23" s="2" t="n">
-        <v>7.99</v>
+        <v>6</v>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
@@ -3982,11 +3982,11 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>TOCINETAS OINK PICANTE 110G</t>
+          <t>Tocino Ahumado Plumrose 250G</t>
         </is>
       </c>
       <c r="C28" s="2" t="n">
-        <v>1.69</v>
+        <v>4.8</v>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
@@ -4515,7 +4515,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Arroz</t>
+          <t>Harinas</t>
         </is>
       </c>
       <c r="F40" s="2" t="n"/>
@@ -4562,7 +4562,7 @@
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>Enlatados</t>
+          <t>Granos</t>
         </is>
       </c>
       <c r="F41" s="2" t="n"/>
@@ -4605,7 +4605,7 @@
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Enlatados</t>
+          <t>Granos</t>
         </is>
       </c>
       <c r="F42" s="2" t="n"/>
@@ -4777,7 +4777,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Arroz</t>
+          <t>Aceites</t>
         </is>
       </c>
       <c r="F46" s="2" t="n"/>
@@ -6035,11 +6035,11 @@
       </c>
       <c r="B75" s="2" t="inlineStr">
         <is>
-          <t>CARBON EL ZULIA 3KG</t>
+          <t>Cerveza Zulia 6 Pack</t>
         </is>
       </c>
       <c r="C75" s="2" t="n">
-        <v>12.6</v>
+        <v>6</v>
       </c>
       <c r="D75" s="2" t="inlineStr">
         <is>
@@ -6078,11 +6078,11 @@
       </c>
       <c r="B76" s="2" t="inlineStr">
         <is>
-          <t>VELON SANTA TERESA PRIMAVERA</t>
+          <t>Ron Santa Teresa Linaje 750ML</t>
         </is>
       </c>
       <c r="C76" s="2" t="n">
-        <v>5.9</v>
+        <v>18</v>
       </c>
       <c r="D76" s="2" t="inlineStr">
         <is>
@@ -6168,11 +6168,11 @@
       </c>
       <c r="B78" s="2" t="inlineStr">
         <is>
-          <t>SALSA DE TOMATE KETCHUP PAMPERO 397G</t>
+          <t>Ron Pampero Aniversario 750ML</t>
         </is>
       </c>
       <c r="C78" s="2" t="n">
-        <v>2.55</v>
+        <v>22</v>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
@@ -6395,11 +6395,11 @@
       </c>
       <c r="B83" s="2" t="inlineStr">
         <is>
-          <t>GUISANTES CON ZANAHORIAS DEL MONTE 411G</t>
+          <t>Vino Tinto Casillero del Diablo 750ML</t>
         </is>
       </c>
       <c r="C83" s="2" t="n">
-        <v>5.89</v>
+        <v>12.5</v>
       </c>
       <c r="D83" s="2" t="inlineStr">
         <is>
@@ -6438,13 +6438,11 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>Vino Blanco Santa Helena</t>
-        </is>
-      </c>
-      <c r="C84" s="2" t="inlineStr">
-        <is>
-          <t>$8.50</t>
-        </is>
+          <t>Vino Blanco Santa Helena 750ML</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="n">
+        <v>8.5</v>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>

</xml_diff>